<commit_message>
nova versão de produção
</commit_message>
<xml_diff>
--- a/SaidaRPA/Excel/indicador-distribuidora_01-01-2026_31-01-2026.xlsx
+++ b/SaidaRPA/Excel/indicador-distribuidora_01-01-2026_31-01-2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,46 +481,46 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>CEA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Risco a Imagem</t>
+          <t>Imprensa | Notícias de Impacto Negativo</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>CEEE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tratativas detratores</t>
+          <t>Imprensa | Notícias de Impacto Negativo</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CEA</t>
+          <t>CEEE</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Imprensa | Notícias de Impacto Negativo</t>
+          <t>Fila INS Cliente</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -531,67 +531,67 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Imprensa | Notícias de Impacto Negativo</t>
+          <t>Imprensa | Favorabilidade</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>45</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CEEE</t>
+          <t>CSA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Fila INS Cliente</t>
+          <t>Imprensa | Notícias de Impacto Negativo</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CEEE</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Tratativas detratores</t>
+          <t>Imprensa | Notícias de Impacto Negativo</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CEEE</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Imprensa | Favorabilidade</t>
+          <t>Fila INS Cliente</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CEEE</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Rechamadas</t>
+          <t>Imprensa | Favorabilidade</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -601,7 +601,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CSA</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -610,63 +610,63 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Imprensa | Notícias de Impacto Negativo</t>
+          <t>Fila INS Cliente</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>81</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Fila INS Cliente</t>
+          <t>Imprensa | Notícias de Impacto Negativo</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Tratativas detratores</t>
+          <t>Fila INS Cliente</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Imprensa | Favorabilidade</t>
+          <t>Redes Sociais | Menções Negativas</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -676,7 +676,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -685,13 +685,13 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>34</v>
+        <v>98</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -700,142 +700,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Tratativas detratores</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Comportamento Inadequado</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Imprensa | Notícias de Impacto Negativo</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Fila INS Cliente</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Redes Sociais | Menções Negativas</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Tratativas detratores</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>PI</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Imprensa | Notícias de Impacto Negativo</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>PI</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Fila INS Cliente</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
         <v>7</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>PI</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Tratativas detratores</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>